<commit_message>
MS Basic Display #1 complete.
</commit_message>
<xml_diff>
--- a/EMail Scraper Test Script v0.1.xlsx
+++ b/EMail Scraper Test Script v0.1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\EMail_scraper\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA35E6D6-96F0-4EA0-A17D-F8641C9B1CAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21172A2A-9363-42E8-BF75-56AAB6A0A6FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D89C3D2A-9F14-4F11-B7B7-DE577937AD45}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="16">
   <si>
     <t>Test</t>
   </si>
@@ -84,8 +84,7 @@
     <t>Fail</t>
   </si>
   <si>
-    <t>Pass:  Counts &gt; 1
-Fail:  Counts = 1 showing, in error.</t>
+    <t>IMAP error: command: SEARCH =&gt; got more than 1000000 bytes</t>
   </si>
 </sst>
 </file>
@@ -477,7 +476,7 @@
   <cols>
     <col min="2" max="2" width="11.5546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="28.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="53.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
@@ -514,7 +513,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -525,11 +524,9 @@
         <v>6</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>15</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="E3" s="3"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
@@ -541,7 +538,9 @@
       <c r="C4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="2"/>
+      <c r="D4" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="E4" s="2"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
@@ -554,7 +553,9 @@
       <c r="C5" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="2"/>
+      <c r="D5" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="E5" s="2"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
@@ -567,7 +568,9 @@
       <c r="C6" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="2"/>
+      <c r="D6" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="E6" s="2"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
@@ -580,8 +583,12 @@
       <c r="C7" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
+      <c r="D7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>15</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Claude create folder Code, snapshot pre-testing.
</commit_message>
<xml_diff>
--- a/EMail Scraper Test Script v0.1.xlsx
+++ b/EMail Scraper Test Script v0.1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\EMail_scraper\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21172A2A-9363-42E8-BF75-56AAB6A0A6FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13618B1A-369F-4F15-99F0-1022E4C7FA48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D89C3D2A-9F14-4F11-B7B7-DE577937AD45}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="43">
   <si>
     <t>Test</t>
   </si>
@@ -84,7 +84,91 @@
     <t>Fail</t>
   </si>
   <si>
-    <t>IMAP error: command: SEARCH =&gt; got more than 1000000 bytes</t>
+    <t>Create Folder</t>
+  </si>
+  <si>
+    <t>Prompt default folder name</t>
+  </si>
+  <si>
+    <t>Confirm button before action.</t>
+  </si>
+  <si>
+    <t>Progress Bar implementation</t>
+  </si>
+  <si>
+    <t>Move ALL Emails from Sender into Folder</t>
+  </si>
+  <si>
+    <t>Create Email Rule for future Emails from Sender</t>
+  </si>
+  <si>
+    <t>Manage History</t>
+  </si>
+  <si>
+    <t>Allow for 3 'Older Than' Date Ranges:
+1.  Keep in Inbox (0-n days)
+2.  Move to "Folder"
+3.  Delete</t>
+  </si>
+  <si>
+    <t>Not required.</t>
+  </si>
+  <si>
+    <t>Check max age in Inbox.</t>
+  </si>
+  <si>
+    <t>Check date range in 'moved to' folder.</t>
+  </si>
+  <si>
+    <t>Check no Emails from Sender over deletion age.</t>
+  </si>
+  <si>
+    <t>Delete All</t>
+  </si>
+  <si>
+    <t>Ensure Confirm Button and Process</t>
+  </si>
+  <si>
+    <t>Ensure Cancel capability before Confirm</t>
+  </si>
+  <si>
+    <t>Ensure all Emails from Sender deleted.</t>
+  </si>
+  <si>
+    <t>Check for a 'future deletions' check box.</t>
+  </si>
+  <si>
+    <t>If 'future deletions' checked, ensure Email rules is created.</t>
+  </si>
+  <si>
+    <t>Check rule working as required (where provable).</t>
+  </si>
+  <si>
+    <t>Test Email Rule (where provable).</t>
+  </si>
+  <si>
+    <t>Unsubscribe</t>
+  </si>
+  <si>
+    <t>Check text wording/formatting when button pressed.</t>
+  </si>
+  <si>
+    <t>Check no effect from button press (where provable).</t>
+  </si>
+  <si>
+    <t>Archive</t>
+  </si>
+  <si>
+    <t>Ensure prompts for archive/zip name and location.</t>
+  </si>
+  <si>
+    <t>Ensure archive/zip contains all Emails from Sender.</t>
+  </si>
+  <si>
+    <t>Restore from archive/zip to prove Save and Restore capability.</t>
+  </si>
+  <si>
+    <t>Ensure text states: there will be no effect on future Emails from this Sender.  Please see other actions…</t>
   </si>
 </sst>
 </file>
@@ -128,7 +212,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -136,6 +220,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -471,11 +561,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10D9BE4A-9A82-4800-9DE5-70D6F0398678}">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.77734375" style="4" customWidth="1"/>
     <col min="5" max="5" width="53.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -486,7 +576,7 @@
       <c r="B1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="5" t="s">
         <v>0</v>
       </c>
       <c r="D1" s="1" t="s">
@@ -503,7 +593,7 @@
       <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="3" t="s">
         <v>4</v>
       </c>
       <c r="D2" s="2" t="s">
@@ -520,7 +610,7 @@
       <c r="B3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D3" s="2" t="s">
@@ -535,7 +625,7 @@
       <c r="B4" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="3" t="s">
         <v>7</v>
       </c>
       <c r="D4" s="2" t="s">
@@ -550,7 +640,7 @@
       <c r="B5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="3" t="s">
         <v>8</v>
       </c>
       <c r="D5" s="2" t="s">
@@ -565,7 +655,7 @@
       <c r="B6" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D6" s="2" t="s">
@@ -580,14 +670,278 @@
       <c r="B7" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="3" t="s">
         <v>10</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E7" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" s="2">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>15</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" s="2">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" s="2">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="2">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A12" s="2">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" s="2">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A14" s="2">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" s="2">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" s="2">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A17" s="2">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" s="2">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" s="2">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" s="2">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" s="2">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A22" s="2">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A23" s="2">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A24" s="2">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A25" s="2">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A26" s="2">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" s="2">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" s="2">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A29" s="2">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A30" s="2">
+        <v>29</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A31" s="2">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Complete Create Folder for Google with auto-filters
- Gmail API migration (analysis + actions)
- Auto-filter creation working
- 9/12 tests passing
- Known limitations documented
</commit_message>
<xml_diff>
--- a/EMail Scraper Test Script v0.1.xlsx
+++ b/EMail Scraper Test Script v0.1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\EMail_scraper\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13618B1A-369F-4F15-99F0-1022E4C7FA48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94D39268-6D8B-4588-A92C-C1DF4754A52F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D89C3D2A-9F14-4F11-B7B7-DE577937AD45}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="48">
   <si>
     <t>Test</t>
   </si>
@@ -169,6 +169,21 @@
   </si>
   <si>
     <t>Ensure text states: there will be no effect on future Emails from this Sender.  Please see other actions…</t>
+  </si>
+  <si>
+    <t>Omit</t>
+  </si>
+  <si>
+    <t>Work around for MVP</t>
+  </si>
+  <si>
+    <t>Modify</t>
+  </si>
+  <si>
+    <t>Gmails uses Labels, not Folders…  Document features.</t>
+  </si>
+  <si>
+    <t>As we can see Rules that have been created. Severity: 4 not 2.</t>
   </si>
 </sst>
 </file>
@@ -690,6 +705,9 @@
       <c r="C8" s="3" t="s">
         <v>16</v>
       </c>
+      <c r="D8" s="2" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
@@ -701,6 +719,9 @@
       <c r="C9" s="3" t="s">
         <v>17</v>
       </c>
+      <c r="D9" s="2" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
@@ -712,6 +733,12 @@
       <c r="C10" s="3" t="s">
         <v>18</v>
       </c>
+      <c r="D10" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
@@ -723,6 +750,12 @@
       <c r="C11" s="3" t="s">
         <v>19</v>
       </c>
+      <c r="D11" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="12" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
@@ -734,6 +767,9 @@
       <c r="C12" s="3" t="s">
         <v>20</v>
       </c>
+      <c r="D12" s="2" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="2">
@@ -744,6 +780,12 @@
       </c>
       <c r="C13" s="3" t="s">
         <v>34</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Minor tweaks in Delete All testing.
</commit_message>
<xml_diff>
--- a/EMail Scraper Test Script v0.1.xlsx
+++ b/EMail Scraper Test Script v0.1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\EMail_scraper\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94D39268-6D8B-4588-A92C-C1DF4754A52F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DADCA55A-4F38-477A-9430-8D55CFFB4065}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D89C3D2A-9F14-4F11-B7B7-DE577937AD45}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="53">
   <si>
     <t>Test</t>
   </si>
@@ -184,6 +184,21 @@
   </si>
   <si>
     <t>As we can see Rules that have been created. Severity: 4 not 2.</t>
+  </si>
+  <si>
+    <t>Concern about accuracy of counts, but works in principle.</t>
+  </si>
+  <si>
+    <t>Sight checked based on date criteria</t>
+  </si>
+  <si>
+    <t>Sight checked</t>
+  </si>
+  <si>
+    <t>Failed</t>
+  </si>
+  <si>
+    <t>CR:  temporal activity not possible.</t>
   </si>
 </sst>
 </file>
@@ -798,6 +813,12 @@
       <c r="C14" s="4" t="s">
         <v>22</v>
       </c>
+      <c r="D14" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="2">
@@ -809,6 +830,12 @@
       <c r="C15" s="4" t="s">
         <v>24</v>
       </c>
+      <c r="D15" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="2">
@@ -820,8 +847,14 @@
       <c r="C16" s="4" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="D16" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -831,8 +864,14 @@
       <c r="C17" s="4" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D17" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -842,8 +881,11 @@
       <c r="C18" s="4" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D18" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -854,7 +896,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -865,7 +907,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -876,7 +918,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -887,7 +929,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A23" s="2">
         <v>22</v>
       </c>
@@ -898,7 +940,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -909,7 +951,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A25" s="2">
         <v>24</v>
       </c>
@@ -920,7 +962,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A26" s="2">
         <v>25</v>
       </c>
@@ -931,7 +973,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" s="2">
         <v>26</v>
       </c>
@@ -942,7 +984,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" s="2">
         <v>27</v>
       </c>
@@ -953,7 +995,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A29" s="2">
         <v>28</v>
       </c>
@@ -964,7 +1006,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A30" s="2">
         <v>29</v>
       </c>
@@ -975,7 +1017,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A31" s="2">
         <v>30</v>
       </c>

</xml_diff>

<commit_message>
Pre Snapshot backend of Archieve WIP.
</commit_message>
<xml_diff>
--- a/EMail Scraper Test Script v0.1.xlsx
+++ b/EMail Scraper Test Script v0.1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\EMail_scraper\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DADCA55A-4F38-477A-9430-8D55CFFB4065}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07BE8CC1-0C48-4B18-A6F6-AB1A63B362E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D89C3D2A-9F14-4F11-B7B7-DE577937AD45}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="55">
   <si>
     <t>Test</t>
   </si>
@@ -199,6 +199,12 @@
   </si>
   <si>
     <t>CR:  temporal activity not possible.</t>
+  </si>
+  <si>
+    <t>Pending</t>
+  </si>
+  <si>
+    <t>We can see the rule, so test down-prioritised.</t>
   </si>
 </sst>
 </file>
@@ -895,6 +901,9 @@
       <c r="C19" s="4" t="s">
         <v>29</v>
       </c>
+      <c r="D19" s="2" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="2">
@@ -906,6 +915,9 @@
       <c r="C20" s="4" t="s">
         <v>30</v>
       </c>
+      <c r="D20" s="2" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="2">
@@ -917,6 +929,9 @@
       <c r="C21" s="4" t="s">
         <v>31</v>
       </c>
+      <c r="D21" s="2" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="22" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A22" s="2">
@@ -928,6 +943,9 @@
       <c r="C22" s="4" t="s">
         <v>32</v>
       </c>
+      <c r="D22" s="2" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="23" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A23" s="2">
@@ -938,6 +956,12 @@
       </c>
       <c r="C23" s="4" t="s">
         <v>33</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Intra MS OAuth debugging snapshot.
</commit_message>
<xml_diff>
--- a/EMail Scraper Test Script v0.1.xlsx
+++ b/EMail Scraper Test Script v0.1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\EMail_scraper\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07BE8CC1-0C48-4B18-A6F6-AB1A63B362E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F784089-9C62-498F-949C-21E08A886F1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D89C3D2A-9F14-4F11-B7B7-DE577937AD45}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="60">
   <si>
     <t>Test</t>
   </si>
@@ -205,6 +205,21 @@
   </si>
   <si>
     <t>We can see the rule, so test down-prioritised.</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Design Change.  Just creating MyArchive label for MVP</t>
+  </si>
+  <si>
+    <t>Re-design for rule creation implemented and working correctly.</t>
+  </si>
+  <si>
+    <t>Google</t>
+  </si>
+  <si>
+    <t>Microsoft</t>
   </si>
 </sst>
 </file>
@@ -248,7 +263,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -262,6 +277,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -597,462 +618,656 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10D9BE4A-9A82-4800-9DE5-70D6F0398678}">
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="13.88671875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="34.77734375" style="4" customWidth="1"/>
-    <col min="5" max="5" width="53.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="0" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="53.5546875" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="53.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="D1" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="G1" s="6"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="2">
+      <c r="F2" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G2" s="7" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" s="3"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+        <v>55</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="G3" s="3"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E4" s="2"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E4" s="3"/>
+      <c r="F4" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="G4" s="3"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E5" s="2"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F5" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="G5" s="2"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E6" s="2"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F6" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" s="2"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C7" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G7" s="2"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" s="2">
+        <v>6</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D8" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E8" s="2" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="2">
+      <c r="F8" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="G8" s="2"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" s="2">
         <v>7</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="2">
-        <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>15</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>15</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>15</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+        <v>44</v>
+      </c>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>15</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+        <v>45</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+    </row>
+    <row r="13" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A13" s="2">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>15</v>
       </c>
       <c r="C13" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14" s="2">
+        <v>12</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C14" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="D14" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="E13" s="2" t="s">
+      <c r="E14" s="2" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="2">
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+    </row>
+    <row r="15" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A15" s="2">
         <v>13</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" s="2">
-        <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+        <v>48</v>
+      </c>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="2">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="2">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C17" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="F17" s="2"/>
+      <c r="G17" s="2"/>
+    </row>
+    <row r="18" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A18" s="2">
+        <v>16</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C18" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="D18" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="E17" s="2" t="s">
+      <c r="E18" s="2" t="s">
         <v>52</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="2">
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A19" s="2">
         <v>17</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A19" s="2">
-        <v>18</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>27</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F19" s="2"/>
+      <c r="G19" s="2"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="2">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>27</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F20" s="2"/>
+      <c r="G20" s="2"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="2">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>27</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="F21" s="2"/>
+      <c r="G21" s="2"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="2">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>27</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="F22" s="2"/>
+      <c r="G22" s="2"/>
+    </row>
+    <row r="23" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A23" s="2">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>27</v>
       </c>
       <c r="C23" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F23" s="2"/>
+      <c r="G23" s="2"/>
+    </row>
+    <row r="24" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A24" s="2">
+        <v>22</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C24" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="D23" s="2" t="s">
+      <c r="D24" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="E23" s="2" t="s">
+      <c r="E24" s="2" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A24" s="2">
+      <c r="F24" s="2"/>
+      <c r="G24" s="2"/>
+    </row>
+    <row r="25" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A25" s="2">
         <v>23</v>
-      </c>
-      <c r="B24" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A25" s="2">
-        <v>24</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>35</v>
       </c>
       <c r="C25" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="F25" s="2"/>
+      <c r="G25" s="2"/>
+    </row>
+    <row r="26" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A26" s="2">
+        <v>24</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C26" s="4" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A26" s="2">
+      <c r="F26" s="2"/>
+      <c r="G26" s="2"/>
+    </row>
+    <row r="27" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A27" s="2">
         <v>25</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A27" s="2">
-        <v>26</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>38</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+        <v>39</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="F27" s="2"/>
+      <c r="G27" s="2"/>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="2">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>38</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+        <v>28</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F28" s="2"/>
+      <c r="G28" s="2"/>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" s="2">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>38</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+        <v>29</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F29" s="2"/>
+      <c r="G29" s="2"/>
+    </row>
+    <row r="30" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A30" s="2">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>38</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+        <v>40</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F30" s="2"/>
+      <c r="G30" s="2"/>
+    </row>
+    <row r="31" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A31" s="2">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>38</v>
       </c>
       <c r="C31" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F31" s="2"/>
+      <c r="G31" s="2"/>
+    </row>
+    <row r="32" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A32" s="2">
+        <v>30</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C32" s="4" t="s">
         <v>42</v>
       </c>
+      <c r="D32" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="F32" s="2"/>
+      <c r="G32" s="2"/>
+    </row>
+    <row r="33" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F33" s="2"/>
+      <c r="G33" s="2"/>
+    </row>
+    <row r="34" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F34" s="2"/>
+      <c r="G34" s="2"/>
+    </row>
+    <row r="35" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F35" s="2"/>
+      <c r="G35" s="2"/>
+    </row>
+    <row r="36" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F36" s="2"/>
+      <c r="G36" s="2"/>
+    </row>
+    <row r="37" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F37" s="2"/>
+      <c r="G37" s="2"/>
+    </row>
+    <row r="38" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F38" s="2"/>
+      <c r="G38" s="2"/>
+    </row>
+    <row r="39" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F39" s="2"/>
+      <c r="G39" s="2"/>
+    </row>
+    <row r="40" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F40" s="2"/>
+      <c r="G40" s="2"/>
+    </row>
+    <row r="41" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F41" s="2"/>
+      <c r="G41" s="2"/>
+    </row>
+    <row r="42" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F42" s="2"/>
+      <c r="G42" s="2"/>
+    </row>
+    <row r="43" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F43" s="2"/>
+      <c r="G43" s="2"/>
+    </row>
+    <row r="44" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F44" s="2"/>
+      <c r="G44" s="2"/>
+    </row>
+    <row r="45" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F45" s="2"/>
+      <c r="G45" s="2"/>
+    </row>
+    <row r="46" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F46" s="2"/>
+      <c r="G46" s="2"/>
+    </row>
+    <row r="47" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F47" s="2"/>
+      <c r="G47" s="2"/>
+    </row>
+    <row r="48" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F48" s="2"/>
+      <c r="G48" s="2"/>
+    </row>
+    <row r="49" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F49" s="2"/>
+      <c r="G49" s="2"/>
+    </row>
+    <row r="50" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F50" s="2"/>
+      <c r="G50" s="2"/>
+    </row>
+    <row r="51" spans="6:7" x14ac:dyDescent="0.3">
+      <c r="F51" s="2"/>
+      <c r="G51" s="2"/>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="F1:G1"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Fully refactored app.py with simplified OAuth.  Pre-test.  WIP.
</commit_message>
<xml_diff>
--- a/EMail Scraper Test Script v0.1.xlsx
+++ b/EMail Scraper Test Script v0.1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\EMail_scraper\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E537E7C-44BF-4B82-85DB-D0EB5B5AB135}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48DF981C-2FDB-451B-B3AE-F1F54DE317AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D89C3D2A-9F14-4F11-B7B7-DE577937AD45}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="60">
   <si>
     <t>Test</t>
   </si>
@@ -279,10 +279,10 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -629,14 +629,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6" t="s">
+      <c r="E1" s="7"/>
+      <c r="F1" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="G1" s="6"/>
+      <c r="G1" s="7"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -654,10 +654,10 @@
       <c r="E2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="F2" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="G2" s="7" t="s">
+      <c r="G2" s="6" t="s">
         <v>5</v>
       </c>
     </row>
@@ -792,7 +792,9 @@
       <c r="D9" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F9" s="2"/>
+      <c r="F9" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="G9" s="2"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
@@ -808,7 +810,9 @@
       <c r="D10" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F10" s="2"/>
+      <c r="F10" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="G10" s="2"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
@@ -827,7 +831,9 @@
       <c r="E11" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="F11" s="2"/>
+      <c r="F11" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="G11" s="2"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
@@ -846,7 +852,9 @@
       <c r="E12" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="F12" s="2"/>
+      <c r="F12" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="G12" s="2"/>
     </row>
     <row r="13" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">

</xml_diff>